<commit_message>
Matriz: diagonal marcada con guion
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014nvYgaHXNCit5W9mFXrnwi
</commit_message>
<xml_diff>
--- a/docs/Chambea-Matriz-Transiciones.xlsx
+++ b/docs/Chambea-Matriz-Transiciones.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1459" uniqueCount="405">
   <si>
     <t xml:space="preserve">Chambea · Matriz de transiciones entre ocupaciones</t>
   </si>
@@ -692,13 +692,16 @@
     <t xml:space="preserve">Oficio de hoy ↓  /  Podría pasar a →</t>
   </si>
   <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cómo se calcula (igual que el motor de Chambea):</t>
   </si>
   <si>
     <t xml:space="preserve">Proximidad(A → B) = suma de pesos de las habilidades de B que A también tiene ÷ suma de pesos de todas las habilidades de B.</t>
   </si>
   <si>
-    <t xml:space="preserve">No es simétrica: A → B puede ser distinto de B → A, porque cada ocupación pide habilidades con pesos distintos. La diagonal (gris) es la misma ocupación.</t>
+    <t xml:space="preserve">No es simétrica: A → B puede ser distinto de B → A, porque cada ocupación pide habilidades con pesos distintos. La diagonal (—) es la misma ocupación.</t>
   </si>
   <si>
     <t xml:space="preserve">Colores: blanco = no comparten nada · amarillo = comparten algo · verde = muy cercanas.</t>
@@ -801,9 +804,6 @@
   </si>
   <si>
     <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
   </si>
   <si>
     <t xml:space="preserve">Archivo de documentos (habilidad), Registro de datos (habilidad), Computación básica (habilidad), Documentos comerciales (conocimiento), Organización y orden (cualidad), Puntualidad (cualidad), Documentos al día (logro)</t>
@@ -1631,7 +1631,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5075,9 +5075,8 @@
       <c r="B6" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$F$6:$F$49,'Matriz habilidades'!$F$6:$F$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$F$6:$F$49)</f>
-        <v>1</v>
+      <c r="C6" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="D6" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$F$6:$F$49,'Matriz habilidades'!$G$6:$G$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$G$6:$G$49)</f>
@@ -5136,9 +5135,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$G$6:$G$49,'Matriz habilidades'!$F$6:$F$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$F$6:$F$49)</f>
         <v>0.538461538461538</v>
       </c>
-      <c r="D7" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$G$6:$G$49,'Matriz habilidades'!$G$6:$G$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$G$6:$G$49)</f>
-        <v>1</v>
+      <c r="D7" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="E7" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$G$6:$G$49,'Matriz habilidades'!$H$6:$H$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$H$6:$H$49)</f>
@@ -5197,9 +5195,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$H$6:$H$49,'Matriz habilidades'!$G$6:$G$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$G$6:$G$49)</f>
         <v>0.142857142857143</v>
       </c>
-      <c r="E8" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$H$6:$H$49,'Matriz habilidades'!$H$6:$H$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$H$6:$H$49)</f>
-        <v>1</v>
+      <c r="E8" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="F8" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$H$6:$H$49,'Matriz habilidades'!$I$6:$I$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$I$6:$I$49)</f>
@@ -5258,9 +5255,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$I$6:$I$49,'Matriz habilidades'!$H$6:$H$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$H$6:$H$49)</f>
         <v>0.0769230769230769</v>
       </c>
-      <c r="F9" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$I$6:$I$49,'Matriz habilidades'!$I$6:$I$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$I$6:$I$49)</f>
-        <v>1</v>
+      <c r="F9" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="G9" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$I$6:$I$49,'Matriz habilidades'!$J$6:$J$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$J$6:$J$49)</f>
@@ -5319,9 +5315,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$J$6:$J$49,'Matriz habilidades'!$I$6:$I$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$I$6:$I$49)</f>
         <v>0.0769230769230769</v>
       </c>
-      <c r="G10" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$J$6:$J$49,'Matriz habilidades'!$J$6:$J$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$J$6:$J$49)</f>
-        <v>1</v>
+      <c r="G10" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="H10" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$J$6:$J$49,'Matriz habilidades'!$K$6:$K$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$K$6:$K$49)</f>
@@ -5380,9 +5375,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$K$6:$K$49,'Matriz habilidades'!$J$6:$J$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$J$6:$J$49)</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="H11" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$K$6:$K$49,'Matriz habilidades'!$K$6:$K$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$K$6:$K$49)</f>
-        <v>1</v>
+      <c r="H11" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="I11" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$K$6:$K$49,'Matriz habilidades'!$L$6:$L$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$L$6:$L$49)</f>
@@ -5441,9 +5435,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$L$6:$L$49,'Matriz habilidades'!$K$6:$K$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$K$6:$K$49)</f>
         <v>0.0769230769230769</v>
       </c>
-      <c r="I12" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$L$6:$L$49,'Matriz habilidades'!$L$6:$L$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$L$6:$L$49)</f>
-        <v>1</v>
+      <c r="I12" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="J12" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$L$6:$L$49,'Matriz habilidades'!$M$6:$M$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$M$6:$M$49)</f>
@@ -5502,9 +5495,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$M$6:$M$49,'Matriz habilidades'!$L$6:$L$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$L$6:$L$49)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$M$6:$M$49,'Matriz habilidades'!$M$6:$M$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$M$6:$M$49)</f>
-        <v>1</v>
+      <c r="J13" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="K13" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$M$6:$M$49,'Matriz habilidades'!$N$6:$N$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$N$6:$N$49)</f>
@@ -5563,9 +5555,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$N$6:$N$49,'Matriz habilidades'!$M$6:$M$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$M$6:$M$49)</f>
         <v>0.307692307692308</v>
       </c>
-      <c r="K14" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$N$6:$N$49,'Matriz habilidades'!$N$6:$N$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$N$6:$N$49)</f>
-        <v>1</v>
+      <c r="K14" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="L14" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$N$6:$N$49,'Matriz habilidades'!$O$6:$O$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$O$6:$O$49)</f>
@@ -5624,9 +5615,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$O$6:$O$49,'Matriz habilidades'!$N$6:$N$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$N$6:$N$49)</f>
         <v>0.0833333333333333</v>
       </c>
-      <c r="L15" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$O$6:$O$49,'Matriz habilidades'!$O$6:$O$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$O$6:$O$49)</f>
-        <v>1</v>
+      <c r="L15" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="M15" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$O$6:$O$49,'Matriz habilidades'!$P$6:$P$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$P$6:$P$49)</f>
@@ -5685,9 +5675,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$P$6:$P$49,'Matriz habilidades'!$O$6:$O$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$O$6:$O$49)</f>
         <v>0</v>
       </c>
-      <c r="M16" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$P$6:$P$49,'Matriz habilidades'!$P$6:$P$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$P$6:$P$49)</f>
-        <v>1</v>
+      <c r="M16" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="N16" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$P$6:$P$49,'Matriz habilidades'!$Q$6:$Q$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$Q$6:$Q$49)</f>
@@ -5746,9 +5735,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$Q$6:$Q$49,'Matriz habilidades'!$P$6:$P$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$P$6:$P$49)</f>
         <v>0.0714285714285714</v>
       </c>
-      <c r="N17" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$Q$6:$Q$49,'Matriz habilidades'!$Q$6:$Q$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$Q$6:$Q$49)</f>
-        <v>1</v>
+      <c r="N17" s="30" t="s">
+        <v>220</v>
       </c>
       <c r="O17" s="31" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$Q$6:$Q$49,'Matriz habilidades'!$R$6:$R$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$R$6:$R$49)</f>
@@ -5807,29 +5795,28 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$R$6:$R$49,'Matriz habilidades'!$Q$6:$Q$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$Q$6:$Q$49)</f>
         <v>0.166666666666667</v>
       </c>
-      <c r="O18" s="30" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$R$6:$R$49,'Matriz habilidades'!$R$6:$R$49)/SUMPRODUCT('Matriz habilidades'!$E$6:$E$49,'Matriz habilidades'!$R$6:$R$49)</f>
-        <v>1</v>
+      <c r="O18" s="30" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="27" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="32" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="32" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -5873,17 +5860,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>51</v>
@@ -5929,9 +5916,8 @@
       <c r="B6" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$F$6:$F$49,'Matriz habilidades'!$F$6:$F$49)</f>
-        <v>7</v>
+      <c r="C6" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="D6" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$F$6:$F$49,'Matriz habilidades'!$G$6:$G$49)</f>
@@ -5990,9 +5976,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$G$6:$G$49,'Matriz habilidades'!$F$6:$F$49)</f>
         <v>4</v>
       </c>
-      <c r="D7" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$G$6:$G$49,'Matriz habilidades'!$G$6:$G$49)</f>
-        <v>7</v>
+      <c r="D7" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="E7" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$G$6:$G$49,'Matriz habilidades'!$H$6:$H$49)</f>
@@ -6051,9 +6036,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$H$6:$H$49,'Matriz habilidades'!$G$6:$G$49)</f>
         <v>1</v>
       </c>
-      <c r="E8" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$H$6:$H$49,'Matriz habilidades'!$H$6:$H$49)</f>
-        <v>7</v>
+      <c r="E8" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="F8" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$H$6:$H$49,'Matriz habilidades'!$I$6:$I$49)</f>
@@ -6112,9 +6096,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$I$6:$I$49,'Matriz habilidades'!$H$6:$H$49)</f>
         <v>1</v>
       </c>
-      <c r="F9" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$I$6:$I$49,'Matriz habilidades'!$I$6:$I$49)</f>
-        <v>7</v>
+      <c r="F9" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="G9" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$I$6:$I$49,'Matriz habilidades'!$J$6:$J$49)</f>
@@ -6173,9 +6156,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$J$6:$J$49,'Matriz habilidades'!$I$6:$I$49)</f>
         <v>1</v>
       </c>
-      <c r="G10" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$J$6:$J$49,'Matriz habilidades'!$J$6:$J$49)</f>
-        <v>7</v>
+      <c r="G10" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="H10" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$J$6:$J$49,'Matriz habilidades'!$K$6:$K$49)</f>
@@ -6234,9 +6216,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$K$6:$K$49,'Matriz habilidades'!$J$6:$J$49)</f>
         <v>1</v>
       </c>
-      <c r="H11" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$K$6:$K$49,'Matriz habilidades'!$K$6:$K$49)</f>
-        <v>7</v>
+      <c r="H11" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="I11" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$K$6:$K$49,'Matriz habilidades'!$L$6:$L$49)</f>
@@ -6295,9 +6276,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$L$6:$L$49,'Matriz habilidades'!$K$6:$K$49)</f>
         <v>1</v>
       </c>
-      <c r="I12" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$L$6:$L$49,'Matriz habilidades'!$L$6:$L$49)</f>
-        <v>7</v>
+      <c r="I12" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="J12" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$L$6:$L$49,'Matriz habilidades'!$M$6:$M$49)</f>
@@ -6356,9 +6336,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$M$6:$M$49,'Matriz habilidades'!$L$6:$L$49)</f>
         <v>0</v>
       </c>
-      <c r="J13" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$M$6:$M$49,'Matriz habilidades'!$M$6:$M$49)</f>
-        <v>7</v>
+      <c r="J13" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="K13" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$M$6:$M$49,'Matriz habilidades'!$N$6:$N$49)</f>
@@ -6417,9 +6396,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$N$6:$N$49,'Matriz habilidades'!$M$6:$M$49)</f>
         <v>2</v>
       </c>
-      <c r="K14" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$N$6:$N$49,'Matriz habilidades'!$N$6:$N$49)</f>
-        <v>7</v>
+      <c r="K14" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="L14" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$N$6:$N$49,'Matriz habilidades'!$O$6:$O$49)</f>
@@ -6478,9 +6456,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$O$6:$O$49,'Matriz habilidades'!$N$6:$N$49)</f>
         <v>1</v>
       </c>
-      <c r="L15" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$O$6:$O$49,'Matriz habilidades'!$O$6:$O$49)</f>
-        <v>7</v>
+      <c r="L15" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="M15" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$O$6:$O$49,'Matriz habilidades'!$P$6:$P$49)</f>
@@ -6539,9 +6516,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$P$6:$P$49,'Matriz habilidades'!$O$6:$O$49)</f>
         <v>0</v>
       </c>
-      <c r="M16" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$P$6:$P$49,'Matriz habilidades'!$P$6:$P$49)</f>
-        <v>7</v>
+      <c r="M16" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="N16" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$P$6:$P$49,'Matriz habilidades'!$Q$6:$Q$49)</f>
@@ -6600,9 +6576,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$Q$6:$Q$49,'Matriz habilidades'!$P$6:$P$49)</f>
         <v>1</v>
       </c>
-      <c r="N17" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$Q$6:$Q$49,'Matriz habilidades'!$Q$6:$Q$49)</f>
-        <v>7</v>
+      <c r="N17" s="33" t="s">
+        <v>220</v>
       </c>
       <c r="O17" s="34" t="n">
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$Q$6:$Q$49,'Matriz habilidades'!$R$6:$R$49)</f>
@@ -6661,9 +6636,8 @@
         <f aca="false">SUMPRODUCT('Matriz habilidades'!$R$6:$R$49,'Matriz habilidades'!$Q$6:$Q$49)</f>
         <v>2</v>
       </c>
-      <c r="O18" s="33" t="n">
-        <f aca="false">SUMPRODUCT('Matriz habilidades'!$R$6:$R$49,'Matriz habilidades'!$R$6:$R$49)</f>
-        <v>7</v>
+      <c r="O18" s="33" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -6711,12 +6685,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6724,28 +6698,28 @@
         <v>44</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6753,7 +6727,7 @@
         <v>51</v>
       </c>
       <c r="B5" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C5" s="35" t="s">
         <v>52</v>
@@ -6774,10 +6748,10 @@
         <v>56</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I5" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6785,7 +6759,7 @@
         <v>51</v>
       </c>
       <c r="B6" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C6" s="40" t="s">
         <v>53</v>
@@ -6803,13 +6777,13 @@
         <v>3</v>
       </c>
       <c r="G6" s="44" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H6" s="44" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I6" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6817,7 +6791,7 @@
         <v>51</v>
       </c>
       <c r="B7" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C7" s="40" t="s">
         <v>54</v>
@@ -6835,13 +6809,13 @@
         <v>2</v>
       </c>
       <c r="G7" s="44" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H7" s="44" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="I7" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6849,7 +6823,7 @@
         <v>51</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C8" s="40" t="s">
         <v>68</v>
@@ -6867,13 +6841,13 @@
         <v>2</v>
       </c>
       <c r="G8" s="44" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H8" s="44" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I8" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6881,7 +6855,7 @@
         <v>51</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C9" s="40" t="s">
         <v>64</v>
@@ -6902,10 +6876,10 @@
         <v>170</v>
       </c>
       <c r="H9" s="44" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="I9" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6913,7 +6887,7 @@
         <v>51</v>
       </c>
       <c r="B10" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C10" s="40" t="s">
         <v>58</v>
@@ -6934,10 +6908,10 @@
         <v>170</v>
       </c>
       <c r="H10" s="44" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I10" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6945,7 +6919,7 @@
         <v>51</v>
       </c>
       <c r="B11" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C11" s="40" t="s">
         <v>57</v>
@@ -6966,10 +6940,10 @@
         <v>176</v>
       </c>
       <c r="H11" s="44" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I11" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6977,7 +6951,7 @@
         <v>51</v>
       </c>
       <c r="B12" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C12" s="40" t="s">
         <v>63</v>
@@ -6995,13 +6969,13 @@
         <v>0</v>
       </c>
       <c r="G12" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H12" s="44" t="s">
         <v>258</v>
       </c>
       <c r="I12" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7027,13 +7001,13 @@
         <v>0</v>
       </c>
       <c r="G13" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H13" s="44" t="s">
         <v>260</v>
       </c>
       <c r="I13" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7059,13 +7033,13 @@
         <v>0</v>
       </c>
       <c r="G14" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H14" s="44" t="s">
         <v>262</v>
       </c>
       <c r="I14" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7091,13 +7065,13 @@
         <v>0</v>
       </c>
       <c r="G15" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H15" s="44" t="s">
         <v>264</v>
       </c>
       <c r="I15" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7123,13 +7097,13 @@
         <v>0</v>
       </c>
       <c r="G16" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H16" s="44" t="s">
         <v>266</v>
       </c>
       <c r="I16" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7137,7 +7111,7 @@
         <v>52</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C17" s="35" t="s">
         <v>51</v>
@@ -7169,7 +7143,7 @@
         <v>52</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C18" s="40" t="s">
         <v>53</v>
@@ -7187,13 +7161,13 @@
         <v>3</v>
       </c>
       <c r="G18" s="44" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="H18" s="44" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I18" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7201,7 +7175,7 @@
         <v>52</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C19" s="40" t="s">
         <v>57</v>
@@ -7225,7 +7199,7 @@
         <v>270</v>
       </c>
       <c r="I19" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7233,7 +7207,7 @@
         <v>52</v>
       </c>
       <c r="B20" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C20" s="40" t="s">
         <v>54</v>
@@ -7257,7 +7231,7 @@
         <v>271</v>
       </c>
       <c r="I20" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7265,7 +7239,7 @@
         <v>52</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C21" s="40" t="s">
         <v>55</v>
@@ -7289,7 +7263,7 @@
         <v>272</v>
       </c>
       <c r="I21" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7297,7 +7271,7 @@
         <v>52</v>
       </c>
       <c r="B22" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C22" s="40" t="s">
         <v>68</v>
@@ -7321,7 +7295,7 @@
         <v>273</v>
       </c>
       <c r="I22" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7329,7 +7303,7 @@
         <v>52</v>
       </c>
       <c r="B23" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C23" s="40" t="s">
         <v>63</v>
@@ -7347,13 +7321,13 @@
         <v>0</v>
       </c>
       <c r="G23" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H23" s="44" t="s">
         <v>258</v>
       </c>
       <c r="I23" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7361,7 +7335,7 @@
         <v>52</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C24" s="40" t="s">
         <v>60</v>
@@ -7379,13 +7353,13 @@
         <v>0</v>
       </c>
       <c r="G24" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H24" s="44" t="s">
         <v>260</v>
       </c>
       <c r="I24" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7411,13 +7385,13 @@
         <v>0</v>
       </c>
       <c r="G25" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H25" s="44" t="s">
         <v>262</v>
       </c>
       <c r="I25" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7443,13 +7417,13 @@
         <v>0</v>
       </c>
       <c r="G26" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H26" s="44" t="s">
         <v>274</v>
       </c>
       <c r="I26" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7475,13 +7449,13 @@
         <v>0</v>
       </c>
       <c r="G27" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H27" s="44" t="s">
         <v>264</v>
       </c>
       <c r="I27" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7507,13 +7481,13 @@
         <v>0</v>
       </c>
       <c r="G28" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H28" s="44" t="s">
         <v>275</v>
       </c>
       <c r="I28" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7521,7 +7495,7 @@
         <v>55</v>
       </c>
       <c r="B29" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C29" s="35" t="s">
         <v>60</v>
@@ -7545,7 +7519,7 @@
         <v>276</v>
       </c>
       <c r="I29" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7553,7 +7527,7 @@
         <v>55</v>
       </c>
       <c r="B30" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C30" s="40" t="s">
         <v>61</v>
@@ -7577,7 +7551,7 @@
         <v>278</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7585,7 +7559,7 @@
         <v>55</v>
       </c>
       <c r="B31" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C31" s="40" t="s">
         <v>52</v>
@@ -7609,7 +7583,7 @@
         <v>279</v>
       </c>
       <c r="I31" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7617,7 +7591,7 @@
         <v>55</v>
       </c>
       <c r="B32" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C32" s="40" t="s">
         <v>58</v>
@@ -7641,7 +7615,7 @@
         <v>280</v>
       </c>
       <c r="I32" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7649,7 +7623,7 @@
         <v>55</v>
       </c>
       <c r="B33" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C33" s="40" t="s">
         <v>54</v>
@@ -7673,7 +7647,7 @@
         <v>281</v>
       </c>
       <c r="I33" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7681,7 +7655,7 @@
         <v>55</v>
       </c>
       <c r="B34" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C34" s="40" t="s">
         <v>63</v>
@@ -7705,7 +7679,7 @@
         <v>282</v>
       </c>
       <c r="I34" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7713,7 +7687,7 @@
         <v>55</v>
       </c>
       <c r="B35" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C35" s="40" t="s">
         <v>57</v>
@@ -7731,13 +7705,13 @@
         <v>0</v>
       </c>
       <c r="G35" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H35" s="44" t="s">
         <v>283</v>
       </c>
       <c r="I35" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7745,7 +7719,7 @@
         <v>55</v>
       </c>
       <c r="B36" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C36" s="40" t="s">
         <v>67</v>
@@ -7763,13 +7737,13 @@
         <v>0</v>
       </c>
       <c r="G36" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H36" s="44" t="s">
         <v>262</v>
       </c>
       <c r="I36" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7795,7 +7769,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H37" s="44" t="s">
         <v>284</v>
@@ -7827,13 +7801,13 @@
         <v>0</v>
       </c>
       <c r="G38" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H38" s="44" t="s">
         <v>274</v>
       </c>
       <c r="I38" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7859,13 +7833,13 @@
         <v>0</v>
       </c>
       <c r="G39" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H39" s="44" t="s">
         <v>285</v>
       </c>
       <c r="I39" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7891,13 +7865,13 @@
         <v>0</v>
       </c>
       <c r="G40" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H40" s="44" t="s">
         <v>286</v>
       </c>
       <c r="I40" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7905,7 +7879,7 @@
         <v>63</v>
       </c>
       <c r="B41" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C41" s="35" t="s">
         <v>57</v>
@@ -7929,7 +7903,7 @@
         <v>287</v>
       </c>
       <c r="I41" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7937,7 +7911,7 @@
         <v>63</v>
       </c>
       <c r="B42" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C42" s="40" t="s">
         <v>64</v>
@@ -7961,7 +7935,7 @@
         <v>289</v>
       </c>
       <c r="I42" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7969,7 +7943,7 @@
         <v>63</v>
       </c>
       <c r="B43" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C43" s="40" t="s">
         <v>60</v>
@@ -7993,7 +7967,7 @@
         <v>291</v>
       </c>
       <c r="I43" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8001,7 +7975,7 @@
         <v>63</v>
       </c>
       <c r="B44" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C44" s="40" t="s">
         <v>61</v>
@@ -8025,7 +7999,7 @@
         <v>292</v>
       </c>
       <c r="I44" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8033,7 +8007,7 @@
         <v>63</v>
       </c>
       <c r="B45" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C45" s="40" t="s">
         <v>68</v>
@@ -8057,7 +8031,7 @@
         <v>293</v>
       </c>
       <c r="I45" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8065,7 +8039,7 @@
         <v>63</v>
       </c>
       <c r="B46" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C46" s="40" t="s">
         <v>58</v>
@@ -8089,7 +8063,7 @@
         <v>294</v>
       </c>
       <c r="I46" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8097,7 +8071,7 @@
         <v>63</v>
       </c>
       <c r="B47" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C47" s="40" t="s">
         <v>54</v>
@@ -8121,7 +8095,7 @@
         <v>295</v>
       </c>
       <c r="I47" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8129,7 +8103,7 @@
         <v>63</v>
       </c>
       <c r="B48" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C48" s="40" t="s">
         <v>55</v>
@@ -8153,7 +8127,7 @@
         <v>296</v>
       </c>
       <c r="I48" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8179,13 +8153,13 @@
         <v>0</v>
       </c>
       <c r="G49" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H49" s="44" t="s">
         <v>262</v>
       </c>
       <c r="I49" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8211,7 +8185,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H50" s="44" t="s">
         <v>284</v>
@@ -8243,13 +8217,13 @@
         <v>0</v>
       </c>
       <c r="G51" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H51" s="44" t="s">
         <v>286</v>
       </c>
       <c r="I51" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8275,13 +8249,13 @@
         <v>0</v>
       </c>
       <c r="G52" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H52" s="44" t="s">
         <v>297</v>
       </c>
       <c r="I52" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8289,7 +8263,7 @@
         <v>58</v>
       </c>
       <c r="B53" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C53" s="35" t="s">
         <v>64</v>
@@ -8313,7 +8287,7 @@
         <v>298</v>
       </c>
       <c r="I53" s="35" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8321,7 +8295,7 @@
         <v>58</v>
       </c>
       <c r="B54" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C54" s="40" t="s">
         <v>61</v>
@@ -8345,7 +8319,7 @@
         <v>300</v>
       </c>
       <c r="I54" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8353,7 +8327,7 @@
         <v>58</v>
       </c>
       <c r="B55" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C55" s="40" t="s">
         <v>54</v>
@@ -8377,7 +8351,7 @@
         <v>302</v>
       </c>
       <c r="I55" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8385,7 +8359,7 @@
         <v>58</v>
       </c>
       <c r="B56" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C56" s="40" t="s">
         <v>60</v>
@@ -8409,7 +8383,7 @@
         <v>304</v>
       </c>
       <c r="I56" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8417,7 +8391,7 @@
         <v>58</v>
       </c>
       <c r="B57" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C57" s="40" t="s">
         <v>68</v>
@@ -8441,7 +8415,7 @@
         <v>306</v>
       </c>
       <c r="I57" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8449,7 +8423,7 @@
         <v>58</v>
       </c>
       <c r="B58" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C58" s="40" t="s">
         <v>67</v>
@@ -8473,7 +8447,7 @@
         <v>307</v>
       </c>
       <c r="I58" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8481,7 +8455,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C59" s="40" t="s">
         <v>63</v>
@@ -8505,7 +8479,7 @@
         <v>308</v>
       </c>
       <c r="I59" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8513,7 +8487,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C60" s="40" t="s">
         <v>51</v>
@@ -8569,7 +8543,7 @@
         <v>310</v>
       </c>
       <c r="I61" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8595,13 +8569,13 @@
         <v>0</v>
       </c>
       <c r="G62" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H62" s="44" t="s">
         <v>283</v>
       </c>
       <c r="I62" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8627,13 +8601,13 @@
         <v>0</v>
       </c>
       <c r="G63" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H63" s="44" t="s">
         <v>286</v>
       </c>
       <c r="I63" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8659,13 +8633,13 @@
         <v>0</v>
       </c>
       <c r="G64" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H64" s="44" t="s">
         <v>297</v>
       </c>
       <c r="I64" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8673,7 +8647,7 @@
         <v>67</v>
       </c>
       <c r="B65" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C65" s="35" t="s">
         <v>68</v>
@@ -8697,7 +8671,7 @@
         <v>311</v>
       </c>
       <c r="I65" s="35" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8705,7 +8679,7 @@
         <v>67</v>
       </c>
       <c r="B66" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C66" s="40" t="s">
         <v>54</v>
@@ -8729,7 +8703,7 @@
         <v>312</v>
       </c>
       <c r="I66" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8737,7 +8711,7 @@
         <v>67</v>
       </c>
       <c r="B67" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C67" s="40" t="s">
         <v>60</v>
@@ -8761,7 +8735,7 @@
         <v>313</v>
       </c>
       <c r="I67" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8769,7 +8743,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C68" s="40" t="s">
         <v>58</v>
@@ -8793,7 +8767,7 @@
         <v>314</v>
       </c>
       <c r="I68" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8801,7 +8775,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C69" s="40" t="s">
         <v>61</v>
@@ -8825,7 +8799,7 @@
         <v>315</v>
       </c>
       <c r="I69" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8833,7 +8807,7 @@
         <v>67</v>
       </c>
       <c r="B70" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C70" s="40" t="s">
         <v>53</v>
@@ -8857,7 +8831,7 @@
         <v>316</v>
       </c>
       <c r="I70" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8865,7 +8839,7 @@
         <v>67</v>
       </c>
       <c r="B71" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C71" s="40" t="s">
         <v>57</v>
@@ -8883,13 +8857,13 @@
         <v>0</v>
       </c>
       <c r="G71" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H71" s="44" t="s">
         <v>283</v>
       </c>
       <c r="I71" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8897,7 +8871,7 @@
         <v>67</v>
       </c>
       <c r="B72" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C72" s="40" t="s">
         <v>63</v>
@@ -8915,13 +8889,13 @@
         <v>0</v>
       </c>
       <c r="G72" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H72" s="44" t="s">
         <v>258</v>
       </c>
       <c r="I72" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8947,7 +8921,7 @@
         <v>0</v>
       </c>
       <c r="G73" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H73" s="44" t="s">
         <v>284</v>
@@ -8979,13 +8953,13 @@
         <v>0</v>
       </c>
       <c r="G74" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H74" s="44" t="s">
         <v>274</v>
       </c>
       <c r="I74" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9011,13 +8985,13 @@
         <v>0</v>
       </c>
       <c r="G75" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H75" s="44" t="s">
         <v>266</v>
       </c>
       <c r="I75" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9043,13 +9017,13 @@
         <v>0</v>
       </c>
       <c r="G76" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H76" s="44" t="s">
         <v>297</v>
       </c>
       <c r="I76" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9057,7 +9031,7 @@
         <v>53</v>
       </c>
       <c r="B77" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C77" s="35" t="s">
         <v>51</v>
@@ -9089,7 +9063,7 @@
         <v>53</v>
       </c>
       <c r="B78" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C78" s="40" t="s">
         <v>52</v>
@@ -9113,7 +9087,7 @@
         <v>319</v>
       </c>
       <c r="I78" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9121,7 +9095,7 @@
         <v>53</v>
       </c>
       <c r="B79" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C79" s="40" t="s">
         <v>68</v>
@@ -9145,7 +9119,7 @@
         <v>321</v>
       </c>
       <c r="I79" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9153,7 +9127,7 @@
         <v>53</v>
       </c>
       <c r="B80" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C80" s="40" t="s">
         <v>57</v>
@@ -9177,7 +9151,7 @@
         <v>323</v>
       </c>
       <c r="I80" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9185,7 +9159,7 @@
         <v>53</v>
       </c>
       <c r="B81" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C81" s="40" t="s">
         <v>54</v>
@@ -9209,7 +9183,7 @@
         <v>271</v>
       </c>
       <c r="I81" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9217,7 +9191,7 @@
         <v>53</v>
       </c>
       <c r="B82" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C82" s="40" t="s">
         <v>67</v>
@@ -9241,7 +9215,7 @@
         <v>324</v>
       </c>
       <c r="I82" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9249,7 +9223,7 @@
         <v>53</v>
       </c>
       <c r="B83" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C83" s="40" t="s">
         <v>63</v>
@@ -9267,13 +9241,13 @@
         <v>0</v>
       </c>
       <c r="G83" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H83" s="44" t="s">
         <v>258</v>
       </c>
       <c r="I83" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9281,7 +9255,7 @@
         <v>53</v>
       </c>
       <c r="B84" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C84" s="40" t="s">
         <v>60</v>
@@ -9299,13 +9273,13 @@
         <v>0</v>
       </c>
       <c r="G84" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H84" s="44" t="s">
         <v>260</v>
       </c>
       <c r="I84" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9331,13 +9305,13 @@
         <v>0</v>
       </c>
       <c r="G85" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H85" s="44" t="s">
         <v>274</v>
       </c>
       <c r="I85" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9363,13 +9337,13 @@
         <v>0</v>
       </c>
       <c r="G86" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H86" s="44" t="s">
         <v>264</v>
       </c>
       <c r="I86" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9395,13 +9369,13 @@
         <v>0</v>
       </c>
       <c r="G87" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H87" s="44" t="s">
         <v>275</v>
       </c>
       <c r="I87" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9427,13 +9401,13 @@
         <v>0</v>
       </c>
       <c r="G88" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H88" s="44" t="s">
         <v>266</v>
       </c>
       <c r="I88" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9441,7 +9415,7 @@
         <v>60</v>
       </c>
       <c r="B89" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C89" s="35" t="s">
         <v>55</v>
@@ -9465,7 +9439,7 @@
         <v>325</v>
       </c>
       <c r="I89" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9473,7 +9447,7 @@
         <v>60</v>
       </c>
       <c r="B90" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C90" s="40" t="s">
         <v>61</v>
@@ -9497,7 +9471,7 @@
         <v>327</v>
       </c>
       <c r="I90" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9505,7 +9479,7 @@
         <v>60</v>
       </c>
       <c r="B91" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C91" s="40" t="s">
         <v>64</v>
@@ -9529,7 +9503,7 @@
         <v>329</v>
       </c>
       <c r="I91" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9537,7 +9511,7 @@
         <v>60</v>
       </c>
       <c r="B92" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C92" s="40" t="s">
         <v>54</v>
@@ -9561,7 +9535,7 @@
         <v>330</v>
       </c>
       <c r="I92" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9569,7 +9543,7 @@
         <v>60</v>
       </c>
       <c r="B93" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C93" s="40" t="s">
         <v>58</v>
@@ -9593,7 +9567,7 @@
         <v>331</v>
       </c>
       <c r="I93" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9601,7 +9575,7 @@
         <v>60</v>
       </c>
       <c r="B94" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C94" s="40" t="s">
         <v>63</v>
@@ -9625,7 +9599,7 @@
         <v>332</v>
       </c>
       <c r="I94" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9633,7 +9607,7 @@
         <v>60</v>
       </c>
       <c r="B95" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C95" s="40" t="s">
         <v>67</v>
@@ -9657,7 +9631,7 @@
         <v>333</v>
       </c>
       <c r="I95" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9665,7 +9639,7 @@
         <v>60</v>
       </c>
       <c r="B96" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C96" s="40" t="s">
         <v>57</v>
@@ -9689,7 +9663,7 @@
         <v>334</v>
       </c>
       <c r="I96" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9715,7 +9689,7 @@
         <v>0</v>
       </c>
       <c r="G97" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H97" s="44" t="s">
         <v>284</v>
@@ -9747,13 +9721,13 @@
         <v>0</v>
       </c>
       <c r="G98" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H98" s="44" t="s">
         <v>285</v>
       </c>
       <c r="I98" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9779,13 +9753,13 @@
         <v>0</v>
       </c>
       <c r="G99" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H99" s="44" t="s">
         <v>286</v>
       </c>
       <c r="I99" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9811,13 +9785,13 @@
         <v>0</v>
       </c>
       <c r="G100" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H100" s="44" t="s">
         <v>297</v>
       </c>
       <c r="I100" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9825,7 +9799,7 @@
         <v>54</v>
       </c>
       <c r="B101" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C101" s="35" t="s">
         <v>60</v>
@@ -9849,7 +9823,7 @@
         <v>335</v>
       </c>
       <c r="I101" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9857,7 +9831,7 @@
         <v>54</v>
       </c>
       <c r="B102" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C102" s="40" t="s">
         <v>58</v>
@@ -9881,7 +9855,7 @@
         <v>337</v>
       </c>
       <c r="I102" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9889,7 +9863,7 @@
         <v>54</v>
       </c>
       <c r="B103" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C103" s="40" t="s">
         <v>67</v>
@@ -9913,7 +9887,7 @@
         <v>333</v>
       </c>
       <c r="I103" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9921,7 +9895,7 @@
         <v>54</v>
       </c>
       <c r="B104" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C104" s="40" t="s">
         <v>51</v>
@@ -9953,7 +9927,7 @@
         <v>54</v>
       </c>
       <c r="B105" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C105" s="40" t="s">
         <v>64</v>
@@ -9977,7 +9951,7 @@
         <v>340</v>
       </c>
       <c r="I105" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9985,7 +9959,7 @@
         <v>54</v>
       </c>
       <c r="B106" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C106" s="40" t="s">
         <v>68</v>
@@ -10009,7 +9983,7 @@
         <v>306</v>
       </c>
       <c r="I106" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10017,7 +9991,7 @@
         <v>54</v>
       </c>
       <c r="B107" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C107" s="40" t="s">
         <v>53</v>
@@ -10041,7 +10015,7 @@
         <v>341</v>
       </c>
       <c r="I107" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10049,7 +10023,7 @@
         <v>54</v>
       </c>
       <c r="B108" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C108" s="40" t="s">
         <v>52</v>
@@ -10073,7 +10047,7 @@
         <v>342</v>
       </c>
       <c r="I108" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10105,7 +10079,7 @@
         <v>343</v>
       </c>
       <c r="I109" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10137,7 +10111,7 @@
         <v>308</v>
       </c>
       <c r="I110" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10169,7 +10143,7 @@
         <v>310</v>
       </c>
       <c r="I111" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10195,13 +10169,13 @@
         <v>0</v>
       </c>
       <c r="G112" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H112" s="44" t="s">
         <v>283</v>
       </c>
       <c r="I112" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10209,7 +10183,7 @@
         <v>61</v>
       </c>
       <c r="B113" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C113" s="35" t="s">
         <v>60</v>
@@ -10233,7 +10207,7 @@
         <v>344</v>
       </c>
       <c r="I113" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10241,7 +10215,7 @@
         <v>61</v>
       </c>
       <c r="B114" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C114" s="40" t="s">
         <v>64</v>
@@ -10265,7 +10239,7 @@
         <v>346</v>
       </c>
       <c r="I114" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10273,7 +10247,7 @@
         <v>61</v>
       </c>
       <c r="B115" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C115" s="40" t="s">
         <v>58</v>
@@ -10297,7 +10271,7 @@
         <v>331</v>
       </c>
       <c r="I115" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10305,7 +10279,7 @@
         <v>61</v>
       </c>
       <c r="B116" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C116" s="40" t="s">
         <v>55</v>
@@ -10329,7 +10303,7 @@
         <v>348</v>
       </c>
       <c r="I116" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10337,7 +10311,7 @@
         <v>61</v>
       </c>
       <c r="B117" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C117" s="40" t="s">
         <v>54</v>
@@ -10361,7 +10335,7 @@
         <v>281</v>
       </c>
       <c r="I117" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10369,7 +10343,7 @@
         <v>61</v>
       </c>
       <c r="B118" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C118" s="40" t="s">
         <v>63</v>
@@ -10393,7 +10367,7 @@
         <v>282</v>
       </c>
       <c r="I118" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10401,7 +10375,7 @@
         <v>61</v>
       </c>
       <c r="B119" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C119" s="40" t="s">
         <v>67</v>
@@ -10425,7 +10399,7 @@
         <v>349</v>
       </c>
       <c r="I119" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10433,7 +10407,7 @@
         <v>61</v>
       </c>
       <c r="B120" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C120" s="40" t="s">
         <v>57</v>
@@ -10451,13 +10425,13 @@
         <v>0</v>
       </c>
       <c r="G120" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H120" s="44" t="s">
         <v>283</v>
       </c>
       <c r="I120" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10483,7 +10457,7 @@
         <v>0</v>
       </c>
       <c r="G121" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H121" s="44" t="s">
         <v>284</v>
@@ -10515,13 +10489,13 @@
         <v>0</v>
       </c>
       <c r="G122" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H122" s="44" t="s">
         <v>285</v>
       </c>
       <c r="I122" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10547,13 +10521,13 @@
         <v>0</v>
       </c>
       <c r="G123" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H123" s="44" t="s">
         <v>286</v>
       </c>
       <c r="I123" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="124" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10579,13 +10553,13 @@
         <v>0</v>
       </c>
       <c r="G124" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H124" s="44" t="s">
         <v>297</v>
       </c>
       <c r="I124" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="125" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10593,7 +10567,7 @@
         <v>57</v>
       </c>
       <c r="B125" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C125" s="35" t="s">
         <v>63</v>
@@ -10617,7 +10591,7 @@
         <v>350</v>
       </c>
       <c r="I125" s="35" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10625,7 +10599,7 @@
         <v>57</v>
       </c>
       <c r="B126" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C126" s="40" t="s">
         <v>52</v>
@@ -10649,7 +10623,7 @@
         <v>352</v>
       </c>
       <c r="I126" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10657,7 +10631,7 @@
         <v>57</v>
       </c>
       <c r="B127" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C127" s="40" t="s">
         <v>53</v>
@@ -10681,7 +10655,7 @@
         <v>353</v>
       </c>
       <c r="I127" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10689,7 +10663,7 @@
         <v>57</v>
       </c>
       <c r="B128" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C128" s="40" t="s">
         <v>64</v>
@@ -10713,7 +10687,7 @@
         <v>354</v>
       </c>
       <c r="I128" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10721,7 +10695,7 @@
         <v>57</v>
       </c>
       <c r="B129" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C129" s="40" t="s">
         <v>60</v>
@@ -10745,7 +10719,7 @@
         <v>355</v>
       </c>
       <c r="I129" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10753,7 +10727,7 @@
         <v>57</v>
       </c>
       <c r="B130" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C130" s="40" t="s">
         <v>68</v>
@@ -10777,7 +10751,7 @@
         <v>273</v>
       </c>
       <c r="I130" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10785,7 +10759,7 @@
         <v>57</v>
       </c>
       <c r="B131" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C131" s="40" t="s">
         <v>51</v>
@@ -10817,7 +10791,7 @@
         <v>57</v>
       </c>
       <c r="B132" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C132" s="40" t="s">
         <v>67</v>
@@ -10835,13 +10809,13 @@
         <v>0</v>
       </c>
       <c r="G132" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H132" s="44" t="s">
         <v>262</v>
       </c>
       <c r="I132" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10867,13 +10841,13 @@
         <v>0</v>
       </c>
       <c r="G133" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H133" s="44" t="s">
         <v>264</v>
       </c>
       <c r="I133" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10899,13 +10873,13 @@
         <v>0</v>
       </c>
       <c r="G134" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H134" s="44" t="s">
         <v>275</v>
       </c>
       <c r="I134" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10931,13 +10905,13 @@
         <v>0</v>
       </c>
       <c r="G135" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H135" s="44" t="s">
         <v>357</v>
       </c>
       <c r="I135" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10963,13 +10937,13 @@
         <v>0</v>
       </c>
       <c r="G136" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H136" s="44" t="s">
         <v>266</v>
       </c>
       <c r="I136" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10977,7 +10951,7 @@
         <v>68</v>
       </c>
       <c r="B137" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C137" s="35" t="s">
         <v>67</v>
@@ -11001,7 +10975,7 @@
         <v>358</v>
       </c>
       <c r="I137" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11009,7 +10983,7 @@
         <v>68</v>
       </c>
       <c r="B138" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C138" s="40" t="s">
         <v>53</v>
@@ -11033,7 +11007,7 @@
         <v>359</v>
       </c>
       <c r="I138" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11041,7 +11015,7 @@
         <v>68</v>
       </c>
       <c r="B139" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C139" s="40" t="s">
         <v>64</v>
@@ -11065,7 +11039,7 @@
         <v>340</v>
       </c>
       <c r="I139" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11073,7 +11047,7 @@
         <v>68</v>
       </c>
       <c r="B140" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C140" s="40" t="s">
         <v>58</v>
@@ -11097,7 +11071,7 @@
         <v>360</v>
       </c>
       <c r="I140" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11105,7 +11079,7 @@
         <v>68</v>
       </c>
       <c r="B141" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C141" s="40" t="s">
         <v>54</v>
@@ -11129,7 +11103,7 @@
         <v>362</v>
       </c>
       <c r="I141" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11137,7 +11111,7 @@
         <v>68</v>
       </c>
       <c r="B142" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C142" s="40" t="s">
         <v>51</v>
@@ -11169,7 +11143,7 @@
         <v>68</v>
       </c>
       <c r="B143" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C143" s="40" t="s">
         <v>63</v>
@@ -11193,7 +11167,7 @@
         <v>308</v>
       </c>
       <c r="I143" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11201,7 +11175,7 @@
         <v>68</v>
       </c>
       <c r="B144" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C144" s="40" t="s">
         <v>57</v>
@@ -11222,10 +11196,10 @@
         <v>176</v>
       </c>
       <c r="H144" s="44" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="I144" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11257,7 +11231,7 @@
         <v>365</v>
       </c>
       <c r="I145" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11283,13 +11257,13 @@
         <v>0</v>
       </c>
       <c r="G146" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H146" s="44" t="s">
         <v>260</v>
       </c>
       <c r="I146" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11315,13 +11289,13 @@
         <v>0</v>
       </c>
       <c r="G147" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H147" s="44" t="s">
         <v>264</v>
       </c>
       <c r="I147" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11347,13 +11321,13 @@
         <v>0</v>
       </c>
       <c r="G148" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H148" s="44" t="s">
         <v>266</v>
       </c>
       <c r="I148" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11361,7 +11335,7 @@
         <v>64</v>
       </c>
       <c r="B149" s="35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C149" s="35" t="s">
         <v>58</v>
@@ -11385,7 +11359,7 @@
         <v>366</v>
       </c>
       <c r="I149" s="35" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11393,7 +11367,7 @@
         <v>64</v>
       </c>
       <c r="B150" s="40" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C150" s="40" t="s">
         <v>60</v>
@@ -11417,7 +11391,7 @@
         <v>368</v>
       </c>
       <c r="I150" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11425,7 +11399,7 @@
         <v>64</v>
       </c>
       <c r="B151" s="40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C151" s="40" t="s">
         <v>61</v>
@@ -11449,7 +11423,7 @@
         <v>370</v>
       </c>
       <c r="I151" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11457,7 +11431,7 @@
         <v>64</v>
       </c>
       <c r="B152" s="40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C152" s="40" t="s">
         <v>63</v>
@@ -11481,7 +11455,7 @@
         <v>372</v>
       </c>
       <c r="I152" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11489,7 +11463,7 @@
         <v>64</v>
       </c>
       <c r="B153" s="40" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C153" s="40" t="s">
         <v>68</v>
@@ -11513,7 +11487,7 @@
         <v>306</v>
       </c>
       <c r="I153" s="40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11521,7 +11495,7 @@
         <v>64</v>
       </c>
       <c r="B154" s="40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C154" s="40" t="s">
         <v>54</v>
@@ -11545,7 +11519,7 @@
         <v>362</v>
       </c>
       <c r="I154" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11553,7 +11527,7 @@
         <v>64</v>
       </c>
       <c r="B155" s="40" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C155" s="40" t="s">
         <v>57</v>
@@ -11577,7 +11551,7 @@
         <v>334</v>
       </c>
       <c r="I155" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11585,7 +11559,7 @@
         <v>64</v>
       </c>
       <c r="B156" s="40" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C156" s="40" t="s">
         <v>51</v>
@@ -11635,13 +11609,13 @@
         <v>0</v>
       </c>
       <c r="G157" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H157" s="44" t="s">
         <v>262</v>
       </c>
       <c r="I157" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11667,13 +11641,13 @@
         <v>0</v>
       </c>
       <c r="G158" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H158" s="44" t="s">
         <v>286</v>
       </c>
       <c r="I158" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11699,13 +11673,13 @@
         <v>0</v>
       </c>
       <c r="G159" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H159" s="44" t="s">
         <v>266</v>
       </c>
       <c r="I159" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11731,13 +11705,13 @@
         <v>0</v>
       </c>
       <c r="G160" s="44" t="s">
-        <v>257</v>
+        <v>220</v>
       </c>
       <c r="H160" s="44" t="s">
         <v>297</v>
       </c>
       <c r="I160" s="40" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -11943,10 +11917,10 @@
         <v>44</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>401</v>

</xml_diff>